<commit_message>
mise a jour EDT 05032026
</commit_message>
<xml_diff>
--- a/LectioShed7.8/app_data/Souhaits-SA-2025-26SP.xlsx
+++ b/LectioShed7.8/app_data/Souhaits-SA-2025-26SP.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrani/Documents/codage/Valides/Testing/LectioShed6.8/app_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mrani/Documents/codage/Valides/Testing/LectioShed7.8/app_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35C913BE-1FAA-B944-B9E5-C18297450759}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6C3BE2-111D-7642-B7ED-74C111C74BDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="119">
   <si>
     <t>C1</t>
   </si>
@@ -64,9 +64,6 @@
     <t>BOUHSSA</t>
   </si>
   <si>
-    <t>PHYSIQUE NUCLÉAIRE – P5</t>
-  </si>
-  <si>
     <t>HRICHA</t>
   </si>
   <si>
@@ -97,9 +94,6 @@
     <t>EL JOUAD</t>
   </si>
   <si>
-    <t>PHYSIQUE DES MATÉRIAUX – P5</t>
-  </si>
-  <si>
     <t>MIKDAM</t>
   </si>
   <si>
@@ -280,18 +274,9 @@
     <t>Choix2</t>
   </si>
   <si>
-    <t>OPTIQUE PHYSIQUE - P4</t>
-  </si>
-  <si>
     <t>JELLAL</t>
   </si>
   <si>
-    <t>MECANIQUE QUANTIQUE - P4</t>
-  </si>
-  <si>
-    <t>MECANIQUE QUANTIQUE -P4</t>
-  </si>
-  <si>
     <t>PMC</t>
   </si>
   <si>
@@ -331,9 +316,6 @@
     <t>OPTIQUE GEOMETRIQUE - MI</t>
   </si>
   <si>
-    <t>OPTIQUE ONDULATOIRE - P4</t>
-  </si>
-  <si>
     <t>ARCHITECTURE DES RESEAUX</t>
   </si>
   <si>
@@ -346,12 +328,6 @@
     <t>ELECTRICITE - MI</t>
   </si>
   <si>
-    <t>ELECTRONIQUE ANALOGIQUE – P4</t>
-  </si>
-  <si>
-    <t>ELECTRONIQUE NUMERIQUE - P4</t>
-  </si>
-  <si>
     <t>EL KAMOUNE</t>
   </si>
   <si>
@@ -386,17 +362,51 @@
   </si>
   <si>
     <t>PHYSIQUE QUANTIQUE 2</t>
+  </si>
+  <si>
+    <t>OPTIQUE ONDULATOIRE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OPTIQUE ONDULATOIRE </t>
+  </si>
+  <si>
+    <t>ELECTRONIQUE ANALOGIQUE</t>
+  </si>
+  <si>
+    <t>MECANIQUE QUANTIQUE - P</t>
+  </si>
+  <si>
+    <t>ELECTRONIQUE NUMERIQUE - P</t>
+  </si>
+  <si>
+    <t>OPTIQUE PHYSIQUE</t>
+  </si>
+  <si>
+    <t>PHYSIQUE DES MATÉRIAUX – P</t>
+  </si>
+  <si>
+    <t>PHYSIQUE DES MATÉRIAUX</t>
+  </si>
+  <si>
+    <t>PHYSIQUE NUCLÉAIRE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -420,8 +430,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -683,10 +694,10 @@
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="B1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -698,7 +709,7 @@
         <v>2</v>
       </c>
       <c r="F1" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G1" t="s">
         <v>3</v>
@@ -715,10 +726,10 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -730,7 +741,7 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="G2">
         <v>0</v>
@@ -744,10 +755,10 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C3">
         <v>2</v>
@@ -759,7 +770,7 @@
         <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -771,15 +782,15 @@
         <v>1</v>
       </c>
       <c r="J3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C4">
         <v>3</v>
@@ -791,7 +802,7 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G4">
         <v>0</v>
@@ -803,15 +814,15 @@
         <v>1</v>
       </c>
       <c r="J4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
-        <v>57</v>
-      </c>
-      <c r="B5" t="s">
-        <v>104</v>
+        <v>55</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -823,7 +834,7 @@
         <v>2</v>
       </c>
       <c r="F5" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -835,15 +846,15 @@
         <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -855,7 +866,7 @@
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="G6">
         <v>0</v>
@@ -869,23 +880,23 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A7" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s">
+        <v>87</v>
+      </c>
+      <c r="C7">
+        <v>1</v>
+      </c>
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="s">
         <v>92</v>
       </c>
-      <c r="C7">
-        <v>1</v>
-      </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>97</v>
-      </c>
       <c r="G7">
         <v>0</v>
       </c>
@@ -896,7 +907,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.15">
@@ -904,7 +915,7 @@
         <v>9</v>
       </c>
       <c r="B8" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C8">
         <v>3</v>
@@ -915,8 +926,8 @@
       <c r="E8">
         <v>0</v>
       </c>
-      <c r="F8" t="s">
-        <v>10</v>
+      <c r="F8" s="1" t="s">
+        <v>118</v>
       </c>
       <c r="G8">
         <v>0</v>
@@ -930,10 +941,10 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9" t="s">
-        <v>99</v>
+        <v>37</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>111</v>
       </c>
       <c r="C9">
         <v>1</v>
@@ -944,8 +955,8 @@
       <c r="E9">
         <v>4</v>
       </c>
-      <c r="F9" t="s">
-        <v>82</v>
+      <c r="F9" s="1" t="s">
+        <v>115</v>
       </c>
       <c r="G9">
         <v>1</v>
@@ -962,7 +973,7 @@
         <v>7</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C10">
         <v>1</v>
@@ -974,7 +985,7 @@
         <v>1</v>
       </c>
       <c r="F10" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="G10">
         <v>0</v>
@@ -988,10 +999,10 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C11">
         <v>0</v>
@@ -1002,8 +1013,8 @@
       <c r="E11">
         <v>0</v>
       </c>
-      <c r="F11" t="s">
-        <v>99</v>
+      <c r="F11" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="G11">
         <v>0</v>
@@ -1017,10 +1028,10 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B12" t="s">
-        <v>104</v>
+        <v>31</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>112</v>
       </c>
       <c r="C12">
         <v>0</v>
@@ -1044,27 +1055,27 @@
         <v>4</v>
       </c>
       <c r="J12" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A13" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+      <c r="F13" t="s">
         <v>90</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <v>1</v>
-      </c>
-      <c r="F13" t="s">
-        <v>95</v>
       </c>
       <c r="G13">
         <v>0</v>
@@ -1078,10 +1089,10 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A14" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C14">
         <v>0</v>
@@ -1093,7 +1104,7 @@
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="G14">
         <v>0</v>
@@ -1105,15 +1116,15 @@
         <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
       <c r="C15">
         <v>1</v>
@@ -1125,7 +1136,7 @@
         <v>1</v>
       </c>
       <c r="F15" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="G15">
         <v>0</v>
@@ -1137,15 +1148,15 @@
         <v>0</v>
       </c>
       <c r="J15" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A16" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1157,7 +1168,7 @@
         <v>0</v>
       </c>
       <c r="F16" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G16">
         <v>0</v>
@@ -1169,15 +1180,15 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A17" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -1188,8 +1199,8 @@
       <c r="E17">
         <v>1</v>
       </c>
-      <c r="F17" t="s">
-        <v>21</v>
+      <c r="F17" s="1" t="s">
+        <v>116</v>
       </c>
       <c r="G17">
         <v>0</v>
@@ -1203,10 +1214,10 @@
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C18">
         <v>0</v>
@@ -1218,7 +1229,7 @@
         <v>1</v>
       </c>
       <c r="F18" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G18">
         <v>1</v>
@@ -1232,10 +1243,10 @@
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B19" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="C19">
         <v>1</v>
@@ -1247,7 +1258,7 @@
         <v>1</v>
       </c>
       <c r="F19" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="G19">
         <v>0</v>
@@ -1259,15 +1270,15 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A20" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B20" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C20">
         <v>0</v>
@@ -1279,7 +1290,7 @@
         <v>0</v>
       </c>
       <c r="F20" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="G20">
         <v>0</v>
@@ -1293,10 +1304,10 @@
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A21" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B21" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C21">
         <v>0</v>
@@ -1307,8 +1318,8 @@
       <c r="E21">
         <v>0</v>
       </c>
-      <c r="F21" t="s">
-        <v>21</v>
+      <c r="F21" s="1" t="s">
+        <v>117</v>
       </c>
       <c r="G21">
         <v>0</v>
@@ -1320,15 +1331,15 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A22" t="s">
-        <v>51</v>
-      </c>
-      <c r="B22" t="s">
-        <v>105</v>
+        <v>49</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="C22">
         <v>1</v>
@@ -1340,7 +1351,7 @@
         <v>2</v>
       </c>
       <c r="F22" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="G22">
         <v>1</v>
@@ -1352,27 +1363,27 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A23" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B23" t="s">
+        <v>87</v>
+      </c>
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>1</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23" t="s">
         <v>92</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
-      </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23">
-        <v>0</v>
-      </c>
-      <c r="F23" t="s">
-        <v>97</v>
       </c>
       <c r="G23">
         <v>0</v>
@@ -1386,10 +1397,10 @@
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A24" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B24" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C24">
         <v>1</v>
@@ -1401,7 +1412,7 @@
         <v>1</v>
       </c>
       <c r="F24" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G24">
         <v>1</v>
@@ -1413,15 +1424,15 @@
         <v>0</v>
       </c>
       <c r="J24" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A25" t="s">
-        <v>63</v>
-      </c>
-      <c r="B25" t="s">
-        <v>84</v>
+        <v>61</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="C25">
         <v>0</v>
@@ -1433,7 +1444,7 @@
         <v>0</v>
       </c>
       <c r="F25" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="G25">
         <v>0</v>
@@ -1445,47 +1456,47 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26">
+        <v>0</v>
+      </c>
+      <c r="D26">
+        <v>4</v>
+      </c>
+      <c r="E26">
+        <v>0</v>
+      </c>
+      <c r="F26" t="s">
+        <v>90</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26">
+        <v>2</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26" t="s">
         <v>38</v>
-      </c>
-      <c r="B26" t="s">
-        <v>87</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
-      </c>
-      <c r="D26">
-        <v>4</v>
-      </c>
-      <c r="E26">
-        <v>0</v>
-      </c>
-      <c r="F26" t="s">
-        <v>95</v>
-      </c>
-      <c r="G26">
-        <v>0</v>
-      </c>
-      <c r="H26">
-        <v>2</v>
-      </c>
-      <c r="I26">
-        <v>0</v>
-      </c>
-      <c r="J26" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A27" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B27" t="s">
-        <v>84</v>
+        <v>113</v>
       </c>
       <c r="C27">
         <v>1</v>
@@ -1511,42 +1522,42 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A28" t="s">
+        <v>10</v>
+      </c>
+      <c r="B28" t="s">
+        <v>108</v>
+      </c>
+      <c r="C28">
+        <v>1</v>
+      </c>
+      <c r="D28">
+        <v>1</v>
+      </c>
+      <c r="E28">
+        <v>1</v>
+      </c>
+      <c r="F28" t="s">
         <v>11</v>
       </c>
-      <c r="B28" t="s">
-        <v>116</v>
-      </c>
-      <c r="C28">
-        <v>1</v>
-      </c>
-      <c r="D28">
-        <v>1</v>
-      </c>
-      <c r="E28">
-        <v>1</v>
-      </c>
-      <c r="F28" t="s">
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>2</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28" t="s">
         <v>12</v>
-      </c>
-      <c r="G28">
-        <v>0</v>
-      </c>
-      <c r="H28">
-        <v>2</v>
-      </c>
-      <c r="I28">
-        <v>0</v>
-      </c>
-      <c r="J28" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A29" t="s">
-        <v>83</v>
-      </c>
-      <c r="B29" t="s">
-        <v>85</v>
+        <v>80</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -1557,8 +1568,8 @@
       <c r="E29">
         <v>0</v>
       </c>
-      <c r="F29" t="s">
-        <v>84</v>
+      <c r="F29" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G29">
         <v>1</v>
@@ -1572,10 +1583,10 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A30" t="s">
-        <v>71</v>
-      </c>
-      <c r="B30" t="s">
-        <v>99</v>
+        <v>69</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>110</v>
       </c>
       <c r="C30">
         <v>0</v>
@@ -1587,7 +1598,7 @@
         <v>2</v>
       </c>
       <c r="F30" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G30">
         <v>0</v>
@@ -1599,15 +1610,15 @@
         <v>0</v>
       </c>
       <c r="J30" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A31" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B31" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
       <c r="C31">
         <v>1</v>
@@ -1631,15 +1642,15 @@
         <v>4</v>
       </c>
       <c r="J31" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A32" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B32" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -1651,7 +1662,7 @@
         <v>1</v>
       </c>
       <c r="F32" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H32">
         <v>0</v>
@@ -1662,10 +1673,10 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B33" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C33">
         <v>1</v>
@@ -1677,7 +1688,7 @@
         <v>1</v>
       </c>
       <c r="F33" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="G33">
         <v>0</v>
@@ -1689,15 +1700,15 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A34" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B34" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C34">
         <v>1</v>
@@ -1709,7 +1720,7 @@
         <v>1</v>
       </c>
       <c r="F34" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="G34">
         <v>0</v>
@@ -1721,44 +1732,44 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" t="s">
+        <v>82</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>4</v>
+      </c>
+      <c r="E35">
+        <v>0</v>
+      </c>
+      <c r="F35" t="s">
+        <v>21</v>
+      </c>
+      <c r="H35">
+        <v>2</v>
+      </c>
+      <c r="I35">
+        <v>4</v>
+      </c>
+      <c r="J35" t="s">
         <v>22</v>
-      </c>
-      <c r="B35" t="s">
-        <v>87</v>
-      </c>
-      <c r="C35">
-        <v>0</v>
-      </c>
-      <c r="D35">
-        <v>4</v>
-      </c>
-      <c r="E35">
-        <v>0</v>
-      </c>
-      <c r="F35" t="s">
-        <v>23</v>
-      </c>
-      <c r="H35">
-        <v>2</v>
-      </c>
-      <c r="I35">
-        <v>4</v>
-      </c>
-      <c r="J35" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" t="s">
-        <v>88</v>
+        <v>33</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>83</v>
       </c>
       <c r="C36">
         <v>1</v>
@@ -1770,7 +1781,7 @@
         <v>1</v>
       </c>
       <c r="F36" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="G36">
         <v>0</v>
@@ -1782,15 +1793,15 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A37" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C37">
         <v>1</v>
@@ -1802,7 +1813,7 @@
         <v>0</v>
       </c>
       <c r="F37" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="G37">
         <v>0</v>
@@ -1816,10 +1827,10 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A38" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B38" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="C38">
         <v>1</v>
@@ -1831,7 +1842,7 @@
         <v>1</v>
       </c>
       <c r="F38" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
       <c r="G38">
         <v>1</v>
@@ -1843,15 +1854,15 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A39" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B39" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C39">
         <v>0</v>
@@ -1863,7 +1874,7 @@
         <v>0</v>
       </c>
       <c r="F39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="G39">
         <v>0</v>
@@ -1877,10 +1888,10 @@
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B40" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C40">
         <v>0</v>
@@ -1891,8 +1902,8 @@
       <c r="E40">
         <v>0</v>
       </c>
-      <c r="F40" t="s">
-        <v>105</v>
+      <c r="F40" s="1" t="s">
+        <v>114</v>
       </c>
       <c r="G40">
         <v>0</v>
@@ -1906,10 +1917,10 @@
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B41" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="C41">
         <v>3</v>
@@ -1921,7 +1932,7 @@
         <v>0</v>
       </c>
       <c r="F41" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G41">
         <v>0</v>
@@ -1935,10 +1946,10 @@
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A42" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B42" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C42">
         <v>1</v>
@@ -1950,7 +1961,7 @@
         <v>0</v>
       </c>
       <c r="F42" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="G42">
         <v>1</v>
@@ -1962,15 +1973,15 @@
         <v>1</v>
       </c>
       <c r="J42" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A43" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B43" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C43">
         <v>1</v>
@@ -1982,15 +1993,15 @@
         <v>2</v>
       </c>
       <c r="J43" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B44" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C44">
         <v>0</v>
@@ -2002,7 +2013,7 @@
         <v>0</v>
       </c>
       <c r="F44" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G44">
         <v>0</v>
@@ -2016,10 +2027,10 @@
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.15">
       <c r="A45" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B45" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="C45">
         <v>1</v>
@@ -2031,7 +2042,7 @@
         <v>0</v>
       </c>
       <c r="F45" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="G45">
         <v>0</v>
@@ -2043,7 +2054,7 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>